<commit_message>
Remove the "reclassify purchases" re-sync (admin button, endpoints, script)
A one-time July 2026 cleanup for bills booked as expenses before upload-time
classification. It rewrote every company's expenses/assets/stock and reset
payment matching in one go, with no owner sign-off. Upload already requires
expense / asset / stock before a bill is filed, and payment matching keeps
balances current, so it is no longer needed (founder, AI backlog AB-06).

- routers/ledger: resync_finance + helpers and POST /ledger/reclassify-purchases
- routers/admin: POST/GET /admin/reclassify-purchases; admin Maintenance tab
- scripts/reclassify_purchases.py; services/calculated.classify_purchase
- API baseline (-3 routes), admin route count 71 -> 69, tests + feature map
- Tracker: E3-14.18, AB-06 done, Sprint 11 18/18, Epic 3 56/56

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic3_AI_Foundation.xlsx
+++ b/docs/DecisionOS_Epic3_AI_Foundation.xlsx
@@ -962,7 +962,7 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Epic 3 AI Foundation -- ACTIVE SCOPE COMPLETE (55/55). Sprints 1-11 done (S11 = 2026-10-05/06 AI audit: safety fixes, durable Brain, and step 5 calculated-not-AI; the S4 agent was removed as unused), incl. S10 evals+benchmark: golden-set expansion + CI regression gate (E3-10.4) and the model-comparison benchmark harness (E3-10.6, evals/benchmark.py). Real-media items closed via Epic 10 S9: OCR quality (E3-06.1) + Tamil/Tanglish STT accuracy (E3-07.1). Remaining 12 out of active scope: 5 future-scoped (few-shot, feedback loop, per-tenant vocab, Voyage swap, embed-scope) + 7 Dex 'Ask' chips + per-role nav MOVED to Epic 6. Bug found+fixed while testing: BUG-16 (Gemini OCR model gemini-2.5-flash 404).</t>
+          <t>Epic 3 AI Foundation -- ACTIVE SCOPE COMPLETE (56/56). Sprints 1-11 done (S11 = 2026-10-05/06 AI audit: safety fixes, durable Brain, and step 5 calculated-not-AI; the S4 agent was removed as unused), incl. S10 evals+benchmark: golden-set expansion + CI regression gate (E3-10.4) and the model-comparison benchmark harness (E3-10.6, evals/benchmark.py). Real-media items closed via Epic 10 S9: OCR quality (E3-06.1) + Tamil/Tanglish STT accuracy (E3-07.1). Remaining 12 out of active scope: 5 future-scoped (few-shot, feedback loop, per-tenant vocab, Voyage swap, embed-scope) + 7 Dex 'Ask' chips + per-role nav MOVED to Epic 6. Bug found+fixed while testing: BUG-16 (Gemini OCR model gemini-2.5-flash 404).</t>
         </is>
       </c>
     </row>
@@ -1347,12 +1347,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1367,7 +1367,7 @@
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>Dex/Brain read only what the asker may; agent endpoints removed; WhatsApp: live members only, approval -&gt; Desk draft, no auto-filing by default, approve once; Ask redesigned: access follows the data (no word gate), questions reach the record they name, mine/names/open work/leave dates, Rs + no computed money, readable Dex room cards; Desk briefing no longer an AI call; Company Brain durable (Mongo/Qdrant), relevance cut-off, live access, section chunks, linked sources; Qdrant on Railway (private, persistent) wired via QDRANT_URL; Company Brain page (documents + notes in Qdrant, curated by owner + Manage Team); Journal = decision history for decision makers; finance-note leak closed; step 5: category, purchase class, contact/task scores, work coach and leave impact are calculated rules (no AI), /auth/me never calls AI, honest labels</t>
+          <t>Dex/Brain read only what the asker may; agent endpoints removed; WhatsApp: live members only, approval -&gt; Desk draft, no auto-filing by default, approve once; Ask redesigned: access follows the data (no word gate), questions reach the record they name, mine/names/open work/leave dates, Rs + no computed money, readable Dex room cards; Desk briefing no longer an AI call; Company Brain durable (Mongo/Qdrant), relevance cut-off, live access, section chunks, linked sources; Qdrant on Railway (private, persistent) wired via QDRANT_URL; Company Brain page (documents + notes in Qdrant, curated by owner + Manage Team); Journal = decision history for decision makers; finance-note leak closed; step 5: category, purchase class, contact/task scores, work coach and leave impact are calculated rules (no AI), /auth/me never calls AI, honest labels; the cross-company "reclassify purchases" re-sync removed</t>
         </is>
       </c>
     </row>
@@ -1382,7 +1382,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L68"/>
+  <dimension ref="A1:L69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5447,6 +5447,68 @@
       <c r="L68" t="inlineStr">
         <is>
           <t>Yokesh 2026-10-06 ("check the production logs and confirm qdrant indexing then solve the step 5")</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>E3-14.18</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>routers/ledger.py; routers/admin.py; scripts/reclassify_purchases.py (deleted); services/calculated.py; pages/admin/AdminPortal.js + AdminSections.js</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Remove the "Fix Mis-booked Purchases" re-sync (admin button, owner endpoint, script)</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>A one-time July 2026 cleanup for bills booked as expenses before upload-time classification. It rewrote every company's expenses/assets/stock and reset payment matching in one go, with no owner sign-off -- and could only overwrite what owners had chosen since.</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>E3-14.17</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>DONE 2026-10-06 (founder: "no need for the reclassify button"). Removed resync_finance + its helpers, POST /ledger/reclassify-purchases, POST/GET /admin/reclassify-purchases (+ the admin Maintenance tab, which held only that button), scripts/reclassify_purchases.py, and services/calculated.classify_purchase (no caller left). Upload still requires expense / asset / stock before a bill is filed; payment matching keeps balances current. API baseline regenerated (-3 routes).</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>Yokesh 2026-10-06 ("no need for the reclassify button why we needed that ?" / "yes remove it")</t>
         </is>
       </c>
     </row>
@@ -5790,12 +5852,12 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Super-admin only, per-tenant, consent-checked, dry-run report the owner approves.</t>
+          <t>DONE 2026-10-06 (E3-14.18): removed instead of locked down -- the admin button, its endpoints, the owner endpoint and the script are gone (founder: not needed).</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Dex desktop pass: chat layout, readable answers, honest allowance message
- Desktop: composer docks to the bottom (fade in the room colour), thread fills
  the page, orb steps out in a conversation, full-width column, answers scroll
  their question to the top, auto-growing input focused on arrival.
- Opener questions are cards under the composer (phones too).
- Answers: Dex avatar + name; table cells in words (departments, To do/Doing,
  High, 22 Sep, right-aligned numbers); 8 rows then "Show all"; 6 sources then
  "+N more"; refusals as a notice card.
- 402 allowance/budget says what ran out and when it resets (lib/aiLimit reads
  lib/api detail_full) instead of "AI service error".
- Backend: our own 402/451 refusals are not retried on another key or fallback
  model; the refused coroutine is closed.
- tests/test_dex_desktop_pass.py (9). Tracker: E3-14.19, Sprint 11 19/19,
  Epic 3 57/57; AB-13 Ask speed -> next version.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic3_AI_Foundation.xlsx
+++ b/docs/DecisionOS_Epic3_AI_Foundation.xlsx
@@ -962,11 +962,10 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Epic 3 AI Foundation -- ACTIVE SCOPE COMPLETE (56/56). Sprints 1-11 done (S11 = 2026-10-05/06 AI audit: safety fixes, durable Brain, and step 5 calculated-not-AI; the S4 agent was removed as unused), incl. S10 evals+benchmark: golden-set expansion + CI regression gate (E3-10.4) and the model-comparison benchmark harness (E3-10.6, evals/benchmark.py). Real-media items closed via Epic 10 S9: OCR quality (E3-06.1) + Tamil/Tanglish STT accuracy (E3-07.1). Remaining 12 out of active scope: 5 future-scoped (few-shot, feedback loop, per-tenant vocab, Voyage swap, embed-scope) + 7 Dex 'Ask' chips + per-role nav MOVED to Epic 6. Bug found+fixed while testing: BUG-16 (Gemini OCR model gemini-2.5-flash 404).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4"/>
+          <t>Epic 3 AI Foundation -- ACTIVE SCOPE COMPLETE (57/57). Sprints 1-11 done (S11 = 2026-10-05/06 AI audit: safety fixes, durable Brain, and step 5 calculated-not-AI; the S4 agent was removed as unused), incl. S10 evals+benchmark: golden-set expansion + CI regression gate (E3-10.4) and the model-comparison benchmark harness (E3-10.6, evals/benchmark.py). Real-media items closed via Epic 10 S9: OCR quality (E3-06.1) + Tamil/Tanglish STT accuracy (E3-07.1). Remaining 12 out of active scope: 5 future-scoped (few-shot, feedback loop, per-tenant vocab, Voyage swap, embed-scope) + 7 Dex 'Ask' chips + per-role nav MOVED to Epic 6. Bug found+fixed while testing: BUG-16 (Gemini OCR model gemini-2.5-flash 404).</t>
+        </is>
+      </c>
+    </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
@@ -1347,12 +1346,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1367,7 +1366,7 @@
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>Dex/Brain read only what the asker may; agent endpoints removed; WhatsApp: live members only, approval -&gt; Desk draft, no auto-filing by default, approve once; Ask redesigned: access follows the data (no word gate), questions reach the record they name, mine/names/open work/leave dates, Rs + no computed money, readable Dex room cards; Desk briefing no longer an AI call; Company Brain durable (Mongo/Qdrant), relevance cut-off, live access, section chunks, linked sources; Qdrant on Railway (private, persistent) wired via QDRANT_URL; Company Brain page (documents + notes in Qdrant, curated by owner + Manage Team); Journal = decision history for decision makers; finance-note leak closed; step 5: category, purchase class, contact/task scores, work coach and leave impact are calculated rules (no AI), /auth/me never calls AI, honest labels; the cross-company "reclassify purchases" re-sync removed</t>
+          <t>Dex/Brain read only what the asker may; agent endpoints removed; WhatsApp: live members only, approval -&gt; Desk draft, no auto-filing by default, approve once; Ask redesigned: access follows the data (no word gate), questions reach the record they name, mine/names/open work/leave dates, Rs + no computed money, readable Dex room cards; Desk briefing no longer an AI call; Company Brain durable (Mongo/Qdrant), relevance cut-off, live access, section chunks, linked sources; Qdrant on Railway (private, persistent) wired via QDRANT_URL; Company Brain page (documents + notes in Qdrant, curated by owner + Manage Team); Journal = decision history for decision makers; finance-note leak closed; step 5: category, purchase class, contact/task scores, work coach and leave impact are calculated rules (no AI), /auth/me never calls AI, honest labels; the cross-company "reclassify purchases" re-sync removed; Dex desktop pass (docked chat composer, readable answers, honest allowance message)</t>
         </is>
       </c>
     </row>
@@ -1382,7 +1381,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L69"/>
+  <dimension ref="A1:L70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5509,6 +5508,63 @@
       <c r="L69" t="inlineStr">
         <is>
           <t>Yokesh 2026-10-06 ("no need for the reclassify button why we needed that ?" / "yes remove it")</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>E3-14.19</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>pages/Brain.js; pages/brain/DexStage.jsx; pages/AskAI.js; lib/aiLimit.js; integrations/llm.py; services/ai/llm_limits.py</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Dex</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Dex desktop pass: chat layout, readable answers, honest allowance message</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Checked in the browser at desktop width: the opener questions sat at the top of an empty page, far from the input; in a conversation the orb sat between thread and composer, the composer halved in width and scrolled off-screen under a long answer, and the page landed on the END of each answer. Tables printed stored values (sales_&amp;_order_management, todo, in_progress, 2026-09-22 wrapping at the hyphen); 20 sources were 20 chips; "DEX -&gt;" was glued to the first word. A company over its monthly AI allowance read "AI service error. Please try again." (the 402 detail was discarded) while the backend retried the same refusal on a second key and a fallback model.</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>DONE 2026-10-06. Desktop (md+): the composer docks to the bottom of the screen with a fade in the room colour, the thread fills the page above it, the orb steps out once a conversation exists, the column is full width, an answer scrolls its question to the top, the box grows as you type and has focus on arrival. Opener questions are cards under the composer (phones too). Answers: Dex avatar + name; table cells in words (department names, To do/Doing, High, 22 Sep, right-aligned numbers, no wrapped dates); 8 rows then "Show all"; 6 sources then "+N more"; refusals as a notice card. 402 allowance/budget says what ran out and the reset date (lib/aiLimit, reads lib/api detail_full). Backend: 402/451 not retried on other keys/models; refused coroutine closed. tests/test_dex_desktop_pass.py (9). Verified live on scratch (desktop 1024 + phone 375).</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>Yokesh 2026-10-06 ("fix the UI of the desktop dex section ... understand the UX as well")</t>
         </is>
       </c>
     </row>
@@ -6181,12 +6237,12 @@
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Next version</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>Smaller context, stream the answer, cache identical questions.</t>
+          <t>Next version (Yokesh 2026-10-07: "put the ASK speed in the backlogs ai. we will do that in next version"). Plan: stream the answer as it is written, cache identical questions per company, trim the context sent to the answer writer.</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">

</xml_diff>

<commit_message>
AI backlog small fixes: honest finance brief, attachments read not filed, log levels
- AB-14: a finance brief that could not be written (allowance used up, AI
  off, failed call) is no longer cached as "Not enough data yet"; it says why
  in a neutral note, and Refresh does not claim "refreshed" over it.
- AB-15: Ask attachments go to /files and ride the question (file_ids); /ask
  reads only the asker's own files for that answer, cited "Attached". Nothing
  is filed into the Company Brain. Desktop Dex sends a paperclip file with the
  question too.
- AB-18: INFO/WARNING to stdout, ERROR to stderr, so Railway's error view
  shows only errors.
- tests/test_ai_backlog_small_fixes.py (8). Tracker: E3-14.20, AB-14/15/18
  done, Sprint 11 20/20, Epic 3 58/58.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic3_AI_Foundation.xlsx
+++ b/docs/DecisionOS_Epic3_AI_Foundation.xlsx
@@ -962,10 +962,11 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Epic 3 AI Foundation -- ACTIVE SCOPE COMPLETE (57/57). Sprints 1-11 done (S11 = 2026-10-05/06 AI audit: safety fixes, durable Brain, and step 5 calculated-not-AI; the S4 agent was removed as unused), incl. S10 evals+benchmark: golden-set expansion + CI regression gate (E3-10.4) and the model-comparison benchmark harness (E3-10.6, evals/benchmark.py). Real-media items closed via Epic 10 S9: OCR quality (E3-06.1) + Tamil/Tanglish STT accuracy (E3-07.1). Remaining 12 out of active scope: 5 future-scoped (few-shot, feedback loop, per-tenant vocab, Voyage swap, embed-scope) + 7 Dex 'Ask' chips + per-role nav MOVED to Epic 6. Bug found+fixed while testing: BUG-16 (Gemini OCR model gemini-2.5-flash 404).</t>
-        </is>
-      </c>
-    </row>
+          <t>Epic 3 AI Foundation -- ACTIVE SCOPE COMPLETE (58/58). Sprints 1-11 done (S11 = 2026-10-05/06 AI audit: safety fixes, durable Brain, and step 5 calculated-not-AI; the S4 agent was removed as unused), incl. S10 evals+benchmark: golden-set expansion + CI regression gate (E3-10.4) and the model-comparison benchmark harness (E3-10.6, evals/benchmark.py). Real-media items closed via Epic 10 S9: OCR quality (E3-06.1) + Tamil/Tanglish STT accuracy (E3-07.1). Remaining 12 out of active scope: 5 future-scoped (few-shot, feedback loop, per-tenant vocab, Voyage swap, embed-scope) + 7 Dex 'Ask' chips + per-role nav MOVED to Epic 6. Bug found+fixed while testing: BUG-16 (Gemini OCR model gemini-2.5-flash 404).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
@@ -1346,12 +1347,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1366,7 +1367,7 @@
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>Dex/Brain read only what the asker may; agent endpoints removed; WhatsApp: live members only, approval -&gt; Desk draft, no auto-filing by default, approve once; Ask redesigned: access follows the data (no word gate), questions reach the record they name, mine/names/open work/leave dates, Rs + no computed money, readable Dex room cards; Desk briefing no longer an AI call; Company Brain durable (Mongo/Qdrant), relevance cut-off, live access, section chunks, linked sources; Qdrant on Railway (private, persistent) wired via QDRANT_URL; Company Brain page (documents + notes in Qdrant, curated by owner + Manage Team); Journal = decision history for decision makers; finance-note leak closed; step 5: category, purchase class, contact/task scores, work coach and leave impact are calculated rules (no AI), /auth/me never calls AI, honest labels; the cross-company "reclassify purchases" re-sync removed; Dex desktop pass (docked chat composer, readable answers, honest allowance message)</t>
+          <t>Dex/Brain read only what the asker may; agent endpoints removed; WhatsApp: live members only, approval -&gt; Desk draft, no auto-filing by default, approve once; Ask redesigned: access follows the data (no word gate), questions reach the record they name, mine/names/open work/leave dates, Rs + no computed money, readable Dex room cards; Desk briefing no longer an AI call; Company Brain durable (Mongo/Qdrant), relevance cut-off, live access, section chunks, linked sources; Qdrant on Railway (private, persistent) wired via QDRANT_URL; Company Brain page (documents + notes in Qdrant, curated by owner + Manage Team); Journal = decision history for decision makers; finance-note leak closed; step 5: category, purchase class, contact/task scores, work coach and leave impact are calculated rules (no AI), /auth/me never calls AI, honest labels; the cross-company "reclassify purchases" re-sync removed; Dex desktop pass (docked chat composer, readable answers, honest allowance message); AB-14/15/18 small fixes</t>
         </is>
       </c>
     </row>
@@ -1381,7 +1382,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L70"/>
+  <dimension ref="A1:L71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5565,6 +5566,63 @@
       <c r="L70" t="inlineStr">
         <is>
           <t>Yokesh 2026-10-06 ("fix the UI of the desktop dex section ... understand the UX as well")</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>E3-14.20</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>routers/ledger.py; pages/finance/FinanceAi.jsx; routers/brain.py; models/brain.py; hooks/useDexConversation.js; pages/Brain.js; pages/brain/DexStage.jsx; core/__init__.py</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>AI backlog small fixes: honest finance brief, attachments read not filed, log levels</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>AB-14: a brief that failed (allowance, AI off, timeout) was cached as "Not enough data yet" until the figures changed. AB-15: Ask filed every attachment into the Company Brain -- refused for members without Manage Team, permanent for everyone else; desktop Dex ignored a paperclip file when asking. AB-18: every log line went to stderr, which Railway marks "error".</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>DONE 2026-10-07. AB-14: failure -&gt; {unavailable, headline: why}, not stored; panel shows a neutral note. AB-15: /files + AskRequest.file_ids; routers/brain._attached_files reads only the asker's own files (max 3, 6,000 chars each) into the answer as attached_files; a closed-records question still answers from the asker's own file without opening the records; cited "Attached". AB-18: INFO/WARNING -&gt; stdout, ERROR -&gt; stderr. Department names in Dex checked: the page already has the company's own list (earlier note was a refresh-timing mistake). tests/test_ai_backlog_small_fixes.py (8). Verified live on scratch: brief note over the allowance; a bill attached on desktop Dex answered from the file, 0 Brain documents created.</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>Yokesh 2026-10-07 ("first push then do this")</t>
         </is>
       </c>
     </row>
@@ -6284,10 +6342,14 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>Backlog</t>
-        </is>
-      </c>
-      <c r="H15" s="4" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>DONE 2026-10-07 (E3-14.20): a brief that could not be written is not cached; it says why (allowance used up / AI off / failed call) in a neutral note, and Refresh no longer says "refreshed" over it.</t>
+        </is>
+      </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
           <t>Yokesh 2026-10-06 (AI audit follow-up)</t>
@@ -6327,10 +6389,14 @@
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>Backlog</t>
-        </is>
-      </c>
-      <c r="H16" s="4" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>DONE 2026-10-07 (E3-14.20): Ask attachments go to /files and ride the question as file_ids; /ask reads only the asker's own files for that answer (cited "Attached"). Nothing is filed into the Company Brain. Desktop Dex now sends a paperclip file with the question too.</t>
+        </is>
+      </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
           <t>Yokesh 2026-10-06 (AI audit follow-up)</t>
@@ -6460,12 +6526,12 @@
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>Log INFO to stdout.</t>
+          <t>DONE 2026-10-07 (E3-14.20): INFO/WARNING to stdout, ERROR+ to stderr (core._log_handlers).</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">

</xml_diff>

<commit_message>
AB-05: "AI off" stops every AI path, not only Claude's
- services/ai/llm_limits.require_ai_allowed: the company's AI consent is
  checked before any provider call outside guarded_llm (451 when refused;
  no company = nothing to check; a consent read failure fails open).
- Wired into Finance bill reading, document import, image/PDF reading,
  speech-to-text and embeddings (Ask questions were still embedded).
- WhatsApp replies "AI is switched off for your company" / allowance used up
  instead of "please try again"; bill uploads return bill_note saying why the
  bill was not read.
- tests/test_ai_off_everywhere.py (12). Tracker: E3-14.21, AB-05 done,
  Sprint 11 21/21, Epic 3 59/59.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic3_AI_Foundation.xlsx
+++ b/docs/DecisionOS_Epic3_AI_Foundation.xlsx
@@ -962,7 +962,7 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Epic 3 AI Foundation -- ACTIVE SCOPE COMPLETE (58/58). Sprints 1-11 done (S11 = 2026-10-05/06 AI audit: safety fixes, durable Brain, and step 5 calculated-not-AI; the S4 agent was removed as unused), incl. S10 evals+benchmark: golden-set expansion + CI regression gate (E3-10.4) and the model-comparison benchmark harness (E3-10.6, evals/benchmark.py). Real-media items closed via Epic 10 S9: OCR quality (E3-06.1) + Tamil/Tanglish STT accuracy (E3-07.1). Remaining 12 out of active scope: 5 future-scoped (few-shot, feedback loop, per-tenant vocab, Voyage swap, embed-scope) + 7 Dex 'Ask' chips + per-role nav MOVED to Epic 6. Bug found+fixed while testing: BUG-16 (Gemini OCR model gemini-2.5-flash 404).</t>
+          <t>Epic 3 AI Foundation -- ACTIVE SCOPE COMPLETE (59/59). Sprints 1-11 done (S11 = 2026-10-05/06 AI audit: safety fixes, durable Brain, and step 5 calculated-not-AI; the S4 agent was removed as unused), incl. S10 evals+benchmark: golden-set expansion + CI regression gate (E3-10.4) and the model-comparison benchmark harness (E3-10.6, evals/benchmark.py). Real-media items closed via Epic 10 S9: OCR quality (E3-06.1) + Tamil/Tanglish STT accuracy (E3-07.1). Remaining 12 out of active scope: 5 future-scoped (few-shot, feedback loop, per-tenant vocab, Voyage swap, embed-scope) + 7 Dex 'Ask' chips + per-role nav MOVED to Epic 6. Bug found+fixed while testing: BUG-16 (Gemini OCR model gemini-2.5-flash 404).</t>
         </is>
       </c>
     </row>
@@ -1347,12 +1347,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1367,7 +1367,7 @@
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>Dex/Brain read only what the asker may; agent endpoints removed; WhatsApp: live members only, approval -&gt; Desk draft, no auto-filing by default, approve once; Ask redesigned: access follows the data (no word gate), questions reach the record they name, mine/names/open work/leave dates, Rs + no computed money, readable Dex room cards; Desk briefing no longer an AI call; Company Brain durable (Mongo/Qdrant), relevance cut-off, live access, section chunks, linked sources; Qdrant on Railway (private, persistent) wired via QDRANT_URL; Company Brain page (documents + notes in Qdrant, curated by owner + Manage Team); Journal = decision history for decision makers; finance-note leak closed; step 5: category, purchase class, contact/task scores, work coach and leave impact are calculated rules (no AI), /auth/me never calls AI, honest labels; the cross-company "reclassify purchases" re-sync removed; Dex desktop pass (docked chat composer, readable answers, honest allowance message); AB-14/15/18 small fixes</t>
+          <t>Dex/Brain read only what the asker may; agent endpoints removed; WhatsApp: live members only, approval -&gt; Desk draft, no auto-filing by default, approve once; Ask redesigned: access follows the data (no word gate), questions reach the record they name, mine/names/open work/leave dates, Rs + no computed money, readable Dex room cards; Desk briefing no longer an AI call; Company Brain durable (Mongo/Qdrant), relevance cut-off, live access, section chunks, linked sources; Qdrant on Railway (private, persistent) wired via QDRANT_URL; Company Brain page (documents + notes in Qdrant, curated by owner + Manage Team); Journal = decision history for decision makers; finance-note leak closed; step 5: category, purchase class, contact/task scores, work coach and leave impact are calculated rules (no AI), /auth/me never calls AI, honest labels; the cross-company "reclassify purchases" re-sync removed; Dex desktop pass (docked chat composer, readable answers, honest allowance message); AB-14/15/18 small fixes; AB-05 AI off stops every AI path</t>
         </is>
       </c>
     </row>
@@ -1382,7 +1382,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L71"/>
+  <dimension ref="A1:L72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5623,6 +5623,63 @@
       <c r="L71" t="inlineStr">
         <is>
           <t>Yokesh 2026-10-07 ("first push then do this")</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>E3-14.21</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>services/ai/llm_limits.py; routers/ledger.py; services/ingestion.py; services/vision.py; services/transcription.py; integrations/embeddings.py; services/whatsapp.py; pages/finance/FinanceForms.jsx</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Safety</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>"AI off" stops every AI path (AB-05)</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Only Claude calls (guarded_llm) checked the company's AI consent. With AI switched off, Gemini still read bills, documents and images on the company's own key; Sarvam/OpenAI/Whisper still transcribed voice and WhatsApp audio; OpenAI still embedded every Ask question -- company data still left for AI providers after the owner said no (DPDP).</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>DONE 2026-10-07. require_ai_allowed(): the request's company (or one named), its consent checked before any provider call; no company (pre-signup) = nothing to check; a consent READ failure fails open like guarded_llm. Wired into ai_extract_ledger_file, ai_extract_document, ai_read_image_general, _transcribe_audio_full_local and embed_texts. Refusal is the existing 451 the app already explains. WhatsApp: 451 -&gt; "AI is switched off for your company...", 402 -&gt; allowance message (not "please try again"). Bill uploads return bill_note ("AI is switched off, so the bill wasn't read"). Out of scope by design: platform-admin key probes (no company data) and the signup interview voice (no company yet). tests/test_ai_off_everywhere.py (12). Live on scratch with consent revoked: bill saved unread with the note, Ask 451, backend log shows no provider attempt.</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>Yokesh 2026-10-07 ("only do the 1")</t>
         </is>
       </c>
     </row>
@@ -5919,12 +5976,12 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>Gate in integrations (gemini/stt/embeddings) by tenant consent; clear user message; tests per path.</t>
+          <t>DONE 2026-10-07 (E3-14.21): one gate (services/ai/llm_limits.require_ai_allowed) at every AI entry point outside guarded_llm -- Finance bill reading, document import, image/PDF reading, speech-to-text, embeddings. Refusal = the existing 451. WhatsApp replies "AI is switched off for your company" (and the allowance case) instead of "try again"; a bill upload says why it was not read.</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">

</xml_diff>